<commit_message>
Enable Abraham Module 2 practice questions
</commit_message>
<xml_diff>
--- a/banks/life-health/Module 2/Topics 5-6 --History US Health Insurance-Public Insurance-Current Issues_Condensed.xlsx
+++ b/banks/life-health/Module 2/Topics 5-6 --History US Health Insurance-Public Insurance-Current Issues_Condensed.xlsx
@@ -1241,7 +1241,7 @@
     <t>Medicare Advantage enrollees are younger and healthier on average than traditional Medicare enrollees.</t>
   </si>
   <si>
-    <t>Medicare Parts C &amp; D</t>
+    <t>Medicare Parts C \&amp; D</t>
   </si>
   <si>
     <t>Medicare Advantage plans must cover more benefits than traditional Medicare, justifying the higher cost.</t>
@@ -1427,7 +1427,7 @@
     <t>Upcoding in Medicare Advantage is estimated to cost the government approximately \$10-15 billion annually.</t>
   </si>
   <si>
-    <t>According to the lecture, the federal government pays approximately \$300 more per enrollee for the Medicare Advantage (Part C) program than for traditional Medicare (Parts A &amp; B). What explains this overpayment?</t>
+    <t>According to the lecture, the federal government pays approximately \$300 more per enrollee for the Medicare Advantage (Part C) program than for traditional Medicare (Parts A \&amp; B). What explains this overpayment?</t>
   </si>
   <si>
     <t>If a physician accepts Medicare assignment, they cannot balance bill beyond the patient’s required cost-sharing.</t>

</xml_diff>